<commit_message>
tracker: fill 5/7-day MA and MTD% columns for all rows after May 5
Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HoDVqecVBj9mDnoNFdjBsS
</commit_message>
<xml_diff>
--- a/MI_PE_Tracking_System.xlsx
+++ b/MI_PE_Tracking_System.xlsx
@@ -159,7 +159,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -250,6 +250,14 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3846,13 +3854,11 @@
       <c r="D5" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E5" s="5">
-        <f>AVERAGE(B5:B5)</f>
-        <v/>
-      </c>
-      <c r="F5" s="5">
-        <f>AVERAGE(B5:B5)</f>
-        <v/>
+      <c r="E5" s="5" t="n">
+        <v>7109.14</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>7109.14</v>
       </c>
       <c r="G5" s="6">
         <f>(B5-6528.52)/6528.52</f>
@@ -3891,13 +3897,11 @@
         <f>(B6-B5)/B5</f>
         <v/>
       </c>
-      <c r="E6" s="5">
-        <f>AVERAGE(B5:B6)</f>
-        <v/>
-      </c>
-      <c r="F6" s="5">
-        <f>AVERAGE(B5:B6)</f>
-        <v/>
+      <c r="E6" s="5" t="n">
+        <v>7086.58</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>7086.58</v>
       </c>
       <c r="G6" s="6">
         <f>(B6-6528.52)/6528.52</f>
@@ -3936,13 +3940,11 @@
         <f>(B7-B6)/B6</f>
         <v/>
       </c>
-      <c r="E7" s="5">
-        <f>AVERAGE(B5:B7)</f>
-        <v/>
-      </c>
-      <c r="F7" s="5">
-        <f>AVERAGE(B5:B7)</f>
-        <v/>
+      <c r="E7" s="5" t="n">
+        <v>7123.52</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>7123.52</v>
       </c>
       <c r="G7" s="6">
         <f>(B7-6528.52)/6528.52</f>
@@ -3981,13 +3983,11 @@
         <f>(B8-B7)/B7</f>
         <v/>
       </c>
-      <c r="E8" s="5">
-        <f>AVERAGE(B5:B8)</f>
-        <v/>
-      </c>
-      <c r="F8" s="5">
-        <f>AVERAGE(B5:B8)</f>
-        <v/>
+      <c r="E8" s="5" t="n">
+        <v>7108.77</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>7108.77</v>
       </c>
       <c r="G8" s="6">
         <f>(B8-6528.52)/6528.52</f>
@@ -4026,13 +4026,11 @@
         <f>(B9-B8)/B8</f>
         <v/>
       </c>
-      <c r="E9" s="5">
-        <f>AVERAGE(B5:B9)</f>
-        <v/>
-      </c>
-      <c r="F9" s="5">
-        <f>AVERAGE(B5:B9)</f>
-        <v/>
+      <c r="E9" s="5" t="n">
+        <v>7137.11</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>7137.11</v>
       </c>
       <c r="G9" s="6">
         <f>(B9-6528.52)/6528.52</f>
@@ -4071,13 +4069,11 @@
         <f>(B10-B9)/B9</f>
         <v/>
       </c>
-      <c r="E10" s="10">
-        <f>AVERAGE(B6:B10)</f>
-        <v/>
-      </c>
-      <c r="F10" s="10">
-        <f>AVERAGE(B5:B10)</f>
-        <v/>
+      <c r="E10" s="10" t="n">
+        <v>7101.41</v>
+      </c>
+      <c r="F10" s="10" t="n">
+        <v>7123.97</v>
       </c>
       <c r="G10" s="11">
         <f>(B10-6528.52)/6528.52</f>
@@ -4116,13 +4112,11 @@
         <f>(B11-B10)/B10</f>
         <v/>
       </c>
-      <c r="E11" s="10">
-        <f>AVERAGE(B7:B11)</f>
-        <v/>
-      </c>
-      <c r="F11" s="10">
-        <f>AVERAGE(B5:B11)</f>
-        <v/>
+      <c r="E11" s="10" t="n">
+        <v>7155.9</v>
+      </c>
+      <c r="F11" s="10" t="n">
+        <v>7141.52</v>
       </c>
       <c r="G11" s="11">
         <f>(B11-6528.52)/6528.52</f>
@@ -4161,13 +4155,11 @@
         <f>(B12-B11)/B11</f>
         <v/>
       </c>
-      <c r="E12" s="10">
-        <f>AVERAGE(B8:B12)</f>
-        <v/>
-      </c>
-      <c r="F12" s="10">
-        <f>AVERAGE(B6:B12)</f>
-        <v/>
+      <c r="E12" s="10" t="n">
+        <v>7122.17</v>
+      </c>
+      <c r="F12" s="10" t="n">
+        <v>7099.98</v>
       </c>
       <c r="G12" s="11">
         <f>(B12-6528.52)/6528.52</f>
@@ -4206,13 +4198,11 @@
         <f>(B13-B12)/B12</f>
         <v/>
       </c>
-      <c r="E13" s="10">
-        <f>AVERAGE(B9:B13)</f>
-        <v/>
-      </c>
-      <c r="F13" s="10">
-        <f>AVERAGE(B7:B13)</f>
-        <v/>
+      <c r="E13" s="10" t="n">
+        <v>7160.04</v>
+      </c>
+      <c r="F13" s="10" t="n">
+        <v>7146.45</v>
       </c>
       <c r="G13" s="11">
         <f>(B13-6528.52)/6528.52</f>
@@ -4251,13 +4241,11 @@
         <f>(B14-B13)/B13</f>
         <v/>
       </c>
-      <c r="E14" s="10">
-        <f>AVERAGE(B10:B14)</f>
-        <v/>
-      </c>
-      <c r="F14" s="10">
-        <f>AVERAGE(B8:B14)</f>
-        <v/>
+      <c r="E14" s="10" t="n">
+        <v>7184.46</v>
+      </c>
+      <c r="F14" s="10" t="n">
+        <v>7169.26</v>
       </c>
       <c r="G14" s="11">
         <f>(B14-6528.52)/6528.52</f>
@@ -4296,13 +4284,11 @@
         <f>(B15-B14)/B14</f>
         <v/>
       </c>
-      <c r="E15" s="10">
-        <f>AVERAGE(B11:B15)</f>
-        <v/>
-      </c>
-      <c r="F15" s="10">
-        <f>AVERAGE(B9:B15)</f>
-        <v/>
+      <c r="E15" s="10" t="n">
+        <v>7187.33</v>
+      </c>
+      <c r="F15" s="10" t="n">
+        <v>7182.91</v>
       </c>
       <c r="G15" s="11">
         <f>(B15-6528.52)/6528.52</f>
@@ -4341,13 +4327,11 @@
         <f>(B16-B15)/B15</f>
         <v/>
       </c>
-      <c r="E16" s="10">
-        <f>AVERAGE(B12:B16)</f>
-        <v/>
-      </c>
-      <c r="F16" s="10">
-        <f>AVERAGE(B10:B16)</f>
-        <v/>
+      <c r="E16" s="10" t="n">
+        <v>7197.59</v>
+      </c>
+      <c r="F16" s="10" t="n">
+        <v>7199.01</v>
       </c>
       <c r="G16" s="11">
         <f>(B16-6528.52)/6528.52</f>
@@ -4382,9 +4366,15 @@
       <c r="D17" s="18" t="n">
         <v>0.0146</v>
       </c>
-      <c r="E17" s="18" t="n"/>
-      <c r="F17" s="18" t="n"/>
-      <c r="G17" s="18" t="n"/>
+      <c r="E17" s="42" t="n">
+        <v>7242.04</v>
+      </c>
+      <c r="F17" s="42" t="n">
+        <v>7217.15</v>
+      </c>
+      <c r="G17" s="43" t="n">
+        <v>0.0294</v>
+      </c>
       <c r="H17" s="18" t="inlineStr">
         <is>
           <t>BUY</t>
@@ -4412,9 +4402,15 @@
       </c>
       <c r="C18" s="18" t="n"/>
       <c r="D18" s="18" t="n"/>
-      <c r="E18" s="18" t="n"/>
-      <c r="F18" s="18" t="n"/>
-      <c r="G18" s="18" t="n"/>
+      <c r="E18" s="42" t="n">
+        <v>7293.44</v>
+      </c>
+      <c r="F18" s="42" t="n">
+        <v>7251.17</v>
+      </c>
+      <c r="G18" s="43" t="n">
+        <v>0.0359</v>
+      </c>
       <c r="H18" s="18" t="inlineStr">
         <is>
           <t>BUY</t>
@@ -4442,9 +4438,15 @@
       </c>
       <c r="C19" s="18" t="n"/>
       <c r="D19" s="18" t="n"/>
-      <c r="E19" s="18" t="n"/>
-      <c r="F19" s="18" t="n"/>
-      <c r="G19" s="18" t="n"/>
+      <c r="E19" s="42" t="n">
+        <v>7347.7</v>
+      </c>
+      <c r="F19" s="42" t="n">
+        <v>7303.37</v>
+      </c>
+      <c r="G19" s="43" t="n">
+        <v>0.0484</v>
+      </c>
       <c r="H19" s="18" t="inlineStr">
         <is>
           <t>BUY</t>
@@ -4474,9 +4476,15 @@
       <c r="D20" s="18" t="n">
         <v>0.0026</v>
       </c>
-      <c r="E20" s="18" t="n"/>
-      <c r="F20" s="18" t="n"/>
-      <c r="G20" s="18" t="n"/>
+      <c r="E20" s="42" t="n">
+        <v>7427.54</v>
+      </c>
+      <c r="F20" s="42" t="n">
+        <v>7366.94</v>
+      </c>
+      <c r="G20" s="43" t="n">
+        <v>0.0622</v>
+      </c>
       <c r="H20" s="18" t="inlineStr">
         <is>
           <t>BUY</t>
@@ -4506,9 +4514,15 @@
       <c r="D21" s="18" t="n">
         <v>0.0013</v>
       </c>
-      <c r="E21" s="18" t="n"/>
-      <c r="F21" s="18" t="n"/>
-      <c r="G21" s="18" t="n"/>
+      <c r="E21" s="42" t="n">
+        <v>7497.65</v>
+      </c>
+      <c r="F21" s="42" t="n">
+        <v>7421.17</v>
+      </c>
+      <c r="G21" s="43" t="n">
+        <v>0.0013</v>
+      </c>
       <c r="H21" s="18" t="inlineStr">
         <is>
           <t>BUY</t>
@@ -4536,9 +4550,15 @@
       </c>
       <c r="C22" s="41" t="n"/>
       <c r="D22" s="41" t="n"/>
-      <c r="E22" s="41" t="n"/>
-      <c r="F22" s="41" t="n"/>
-      <c r="G22" s="41" t="n"/>
+      <c r="E22" s="44" t="n">
+        <v>7541.42</v>
+      </c>
+      <c r="F22" s="44" t="n">
+        <v>7475.92</v>
+      </c>
+      <c r="G22" s="45" t="n">
+        <v>-0.0021</v>
+      </c>
       <c r="H22" s="41" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -4568,9 +4588,15 @@
       <c r="D23" s="19" t="n">
         <v>-0.0264</v>
       </c>
-      <c r="E23" s="19" t="n"/>
-      <c r="F23" s="19" t="n"/>
-      <c r="G23" s="19" t="n"/>
+      <c r="E23" s="46" t="n">
+        <v>7535.76</v>
+      </c>
+      <c r="F23" s="46" t="n">
+        <v>7493.71</v>
+      </c>
+      <c r="G23" s="47" t="n">
+        <v>-0.0285</v>
+      </c>
       <c r="H23" s="19" t="inlineStr">
         <is>
           <t>SELL</t>
@@ -4602,9 +4628,15 @@
       <c r="D24" s="41" t="n">
         <v>0.003</v>
       </c>
-      <c r="E24" s="41" t="n"/>
-      <c r="F24" s="41" t="n"/>
-      <c r="G24" s="41" t="n"/>
+      <c r="E24" s="44" t="n">
+        <v>7516.63</v>
+      </c>
+      <c r="F24" s="44" t="n">
+        <v>7499.51</v>
+      </c>
+      <c r="G24" s="45" t="n">
+        <v>-0.0256</v>
+      </c>
       <c r="H24" s="41" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -4636,9 +4668,15 @@
       <c r="D25" s="41" t="n">
         <v>-0.0026</v>
       </c>
-      <c r="E25" s="41" t="n"/>
-      <c r="F25" s="41" t="n"/>
-      <c r="G25" s="41" t="n"/>
+      <c r="E25" s="44" t="n">
+        <v>7473.97</v>
+      </c>
+      <c r="F25" s="44" t="n">
+        <v>7495.89</v>
+      </c>
+      <c r="G25" s="45" t="n">
+        <v>-0.0281</v>
+      </c>
       <c r="H25" s="41" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -4670,9 +4708,15 @@
       <c r="D26" s="41" t="n">
         <v>-0.0162</v>
       </c>
-      <c r="E26" s="41" t="n"/>
-      <c r="F26" s="41" t="n"/>
-      <c r="G26" s="41" t="n"/>
+      <c r="E26" s="44" t="n">
+        <v>7405.41</v>
+      </c>
+      <c r="F26" s="44" t="n">
+        <v>7462.4</v>
+      </c>
+      <c r="G26" s="45" t="n">
+        <v>-0.0438</v>
+      </c>
       <c r="H26" s="41" t="inlineStr">
         <is>
           <t>SELL</t>
@@ -4704,9 +4748,15 @@
       <c r="D27" s="41" t="n">
         <v>0.0175</v>
       </c>
-      <c r="E27" s="41" t="n"/>
-      <c r="F27" s="41" t="n"/>
-      <c r="G27" s="41" t="n"/>
+      <c r="E27" s="44" t="n">
+        <v>7367.48</v>
+      </c>
+      <c r="F27" s="44" t="n">
+        <v>7433.02</v>
+      </c>
+      <c r="G27" s="45" t="n">
+        <v>-0.0271</v>
+      </c>
       <c r="H27" s="41" t="inlineStr">
         <is>
           <t>BUY</t>
@@ -4738,9 +4788,15 @@
       <c r="D28" s="41" t="n">
         <v>0.005</v>
       </c>
-      <c r="E28" s="41" t="n"/>
-      <c r="F28" s="41" t="n"/>
-      <c r="G28" s="41" t="n"/>
+      <c r="E28" s="44" t="n">
+        <v>7377.03</v>
+      </c>
+      <c r="F28" s="44" t="n">
+        <v>7407.55</v>
+      </c>
+      <c r="G28" s="45" t="n">
+        <v>-0.0222</v>
+      </c>
       <c r="H28" s="41" t="inlineStr">
         <is>
           <t>BUY</t>
@@ -4772,9 +4828,15 @@
       <c r="D29" s="41" t="n">
         <v>0.0165</v>
       </c>
-      <c r="E29" s="41" t="n"/>
-      <c r="F29" s="41" t="n"/>
-      <c r="G29" s="41" t="n"/>
+      <c r="E29" s="44" t="n">
+        <v>7406.74</v>
+      </c>
+      <c r="F29" s="44" t="n">
+        <v>7403.31</v>
+      </c>
+      <c r="G29" s="45" t="n">
+        <v>-0.006</v>
+      </c>
       <c r="H29" s="41" t="inlineStr">
         <is>
           <t>BUY</t>
@@ -4806,9 +4868,15 @@
       <c r="D30" s="41" t="n">
         <v>-0.0057</v>
       </c>
-      <c r="E30" s="41" t="n"/>
-      <c r="F30" s="41" t="n"/>
-      <c r="G30" s="41" t="n"/>
+      <c r="E30" s="44" t="n">
+        <v>7431.6</v>
+      </c>
+      <c r="F30" s="44" t="n">
+        <v>7421.49</v>
+      </c>
+      <c r="G30" s="45" t="n">
+        <v>-0.0117</v>
+      </c>
       <c r="H30" s="41" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -4838,9 +4906,15 @@
       <c r="D31" s="19" t="n">
         <v>-0.0121</v>
       </c>
-      <c r="E31" s="19" t="n"/>
-      <c r="F31" s="19" t="n"/>
-      <c r="G31" s="19" t="n"/>
+      <c r="E31" s="46" t="n">
+        <v>7462.23</v>
+      </c>
+      <c r="F31" s="46" t="n">
+        <v>7423.54</v>
+      </c>
+      <c r="G31" s="47" t="n">
+        <v>-0.0237</v>
+      </c>
       <c r="H31" s="19" t="inlineStr">
         <is>
           <t>SELL</t>
@@ -4872,9 +4946,15 @@
       <c r="D32" s="19" t="n">
         <v>0.0108</v>
       </c>
-      <c r="E32" s="19" t="n"/>
-      <c r="F32" s="19" t="n"/>
-      <c r="G32" s="19" t="n"/>
+      <c r="E32" s="46" t="n">
+        <v>7483.48</v>
+      </c>
+      <c r="F32" s="46" t="n">
+        <v>7439.81</v>
+      </c>
+      <c r="G32" s="47" t="n">
+        <v>-0.0131</v>
+      </c>
       <c r="H32" s="19" t="inlineStr">
         <is>
           <t>BUY</t>
@@ -4906,6 +4986,15 @@
       <c r="D33" t="n">
         <v>0.0012</v>
       </c>
+      <c r="E33" s="48" t="n">
+        <v>7498.99</v>
+      </c>
+      <c r="F33" s="48" t="n">
+        <v>7474.39</v>
+      </c>
+      <c r="G33" s="49" t="n">
+        <v>-0.012</v>
+      </c>
       <c r="H33" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -4937,6 +5026,15 @@
       <c r="D34" t="n">
         <v>-0.0144</v>
       </c>
+      <c r="E34" s="48" t="n">
+        <v>7461.22</v>
+      </c>
+      <c r="F34" s="48" t="n">
+        <v>7470.27</v>
+      </c>
+      <c r="G34" s="49" t="n">
+        <v>-0.0309</v>
+      </c>
       <c r="H34" t="inlineStr">
         <is>
           <t>SELL</t>
@@ -4968,6 +5066,15 @@
       <c r="D35" t="n">
         <v>-0.001</v>
       </c>
+      <c r="E35" s="48" t="n">
+        <v>7430.67</v>
+      </c>
+      <c r="F35" s="48" t="n">
+        <v>7459.8</v>
+      </c>
+      <c r="G35" s="49" t="n">
+        <v>-0.0318</v>
+      </c>
       <c r="H35" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -4999,6 +5106,15 @@
       <c r="D36" t="n">
         <v>-0.0001</v>
       </c>
+      <c r="E36" s="48" t="n">
+        <v>7418.15</v>
+      </c>
+      <c r="F36" s="48" t="n">
+        <v>7431.69</v>
+      </c>
+      <c r="G36" s="49" t="n">
+        <v>-0.0319</v>
+      </c>
       <c r="H36" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -5027,6 +5143,15 @@
       <c r="D37" t="n">
         <v>0.012</v>
       </c>
+      <c r="E37" s="48" t="n">
+        <v>7407.03</v>
+      </c>
+      <c r="F37" s="48" t="n">
+        <v>7422.26</v>
+      </c>
+      <c r="G37" s="49" t="n">
+        <v>-0.0204</v>
+      </c>
       <c r="H37" t="inlineStr">
         <is>
           <t>BUY</t>
@@ -5058,6 +5183,15 @@
       <c r="D38" t="n">
         <v>0.0003</v>
       </c>
+      <c r="E38" s="48" t="n">
+        <v>7395.11</v>
+      </c>
+      <c r="F38" s="48" t="n">
+        <v>7426.44</v>
+      </c>
+      <c r="G38" s="49" t="n">
+        <v>-0.0198</v>
+      </c>
       <c r="H38" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -5086,6 +5220,15 @@
       <c r="D39" t="n">
         <v>0.0045</v>
       </c>
+      <c r="E39" s="48" t="n">
+        <v>7418.61</v>
+      </c>
+      <c r="F39" s="48" t="n">
+        <v>7423.93</v>
+      </c>
+      <c r="G39" s="49" t="n">
+        <v>0.0045</v>
+      </c>
       <c r="H39" t="inlineStr">
         <is>
           <t>BUY</t>
@@ -5113,6 +5256,15 @@
       </c>
       <c r="D40" t="n">
         <v>-0.0039</v>
+      </c>
+      <c r="E40" s="48" t="n">
+        <v>7437.76</v>
+      </c>
+      <c r="F40" s="48" t="n">
+        <v>7416.07</v>
+      </c>
+      <c r="G40" s="49" t="n">
+        <v>0.0005999999999999999</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
@@ -5143,9 +5295,15 @@
       <c r="D41" s="41" t="n">
         <v>0.0072</v>
       </c>
-      <c r="E41" s="41" t="n"/>
-      <c r="F41" s="41" t="n"/>
-      <c r="G41" s="41" t="n"/>
+      <c r="E41" s="44" t="n">
+        <v>7473.75</v>
+      </c>
+      <c r="F41" s="44" t="n">
+        <v>7440.64</v>
+      </c>
+      <c r="G41" s="45" t="n">
+        <v>0.0118</v>
+      </c>
       <c r="H41" s="41" t="inlineStr">
         <is>
           <t>BUY</t>
@@ -5177,9 +5335,15 @@
       <c r="D42" s="41" t="n">
         <v>-0.0045</v>
       </c>
-      <c r="E42" s="41" t="n"/>
-      <c r="F42" s="41" t="n"/>
-      <c r="G42" s="41" t="n"/>
+      <c r="E42" s="44" t="n">
+        <v>7485.52</v>
+      </c>
+      <c r="F42" s="44" t="n">
+        <v>7461.44</v>
+      </c>
+      <c r="G42" s="45" t="n">
+        <v>0.0073</v>
+      </c>
       <c r="H42" s="41" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -5211,9 +5375,15 @@
       <c r="D43" s="41" t="n">
         <v>-0.0028</v>
       </c>
-      <c r="E43" s="41" t="n"/>
-      <c r="F43" s="41" t="n"/>
-      <c r="G43" s="41" t="n"/>
+      <c r="E43" s="44" t="n">
+        <v>7492.19</v>
+      </c>
+      <c r="F43" s="44" t="n">
+        <v>7479.33</v>
+      </c>
+      <c r="G43" s="45" t="n">
+        <v>0.0045</v>
+      </c>
       <c r="H43" s="41" t="inlineStr">
         <is>
           <t>SELL</t>
@@ -5245,9 +5415,15 @@
       <c r="D44" s="41" t="n">
         <v>0.0081</v>
       </c>
-      <c r="E44" s="41" t="n"/>
-      <c r="F44" s="41" t="n"/>
-      <c r="G44" s="41" t="n"/>
+      <c r="E44" s="44" t="n">
+        <v>7504.32</v>
+      </c>
+      <c r="F44" s="44" t="n">
+        <v>7493.42</v>
+      </c>
+      <c r="G44" s="45" t="n">
+        <v>0.0127</v>
+      </c>
       <c r="H44" s="41" t="inlineStr">
         <is>
           <t>BUY</t>
@@ -5279,9 +5455,15 @@
       <c r="D45" s="41" t="n">
         <v>0.0042</v>
       </c>
-      <c r="E45" s="41" t="n"/>
-      <c r="F45" s="41" t="n"/>
-      <c r="G45" s="41" t="n"/>
+      <c r="E45" s="44" t="n">
+        <v>7528.6</v>
+      </c>
+      <c r="F45" s="44" t="n">
+        <v>7511.43</v>
+      </c>
+      <c r="G45" s="45" t="n">
+        <v>0.0169</v>
+      </c>
       <c r="H45" s="41" t="inlineStr">
         <is>
           <t>BUY</t>
@@ -5313,9 +5495,15 @@
       <c r="D46" s="41" t="n">
         <v>-0.008</v>
       </c>
-      <c r="E46" s="41" t="n"/>
-      <c r="F46" s="41" t="n"/>
-      <c r="G46" s="41" t="n"/>
+      <c r="E46" s="44" t="n">
+        <v>7524.12</v>
+      </c>
+      <c r="F46" s="44" t="n">
+        <v>7516</v>
+      </c>
+      <c r="G46" s="45" t="n">
+        <v>0.008800000000000001</v>
+      </c>
       <c r="H46" s="41" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -5347,9 +5535,15 @@
       <c r="D47" s="41" t="n">
         <v>0.0038</v>
       </c>
-      <c r="E47" s="41" t="n"/>
-      <c r="F47" s="41" t="n"/>
-      <c r="G47" s="41" t="n"/>
+      <c r="E47" s="44" t="n">
+        <v>7532.07</v>
+      </c>
+      <c r="F47" s="44" t="n">
+        <v>7528.81</v>
+      </c>
+      <c r="G47" s="45" t="n">
+        <v>0.0126</v>
+      </c>
       <c r="H47" s="41" t="inlineStr">
         <is>
           <t>BUY</t>
@@ -5381,9 +5575,15 @@
       <c r="D48" s="41" t="n">
         <v>-0.0051</v>
       </c>
-      <c r="E48" s="41" t="n"/>
-      <c r="F48" s="41" t="n"/>
-      <c r="G48" s="41" t="n"/>
+      <c r="E48" s="44" t="n">
+        <v>7542.28</v>
+      </c>
+      <c r="F48" s="44" t="n">
+        <v>7528.28</v>
+      </c>
+      <c r="G48" s="45" t="n">
+        <v>0.0113</v>
+      </c>
       <c r="H48" s="41" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -5443,9 +5643,15 @@
       <c r="D50" s="41" t="n">
         <v>-0.0102</v>
       </c>
-      <c r="E50" s="41" t="n"/>
-      <c r="F50" s="41" t="n"/>
-      <c r="G50" s="41" t="n"/>
+      <c r="E50" s="44" t="n">
+        <v>7524.96</v>
+      </c>
+      <c r="F50" s="44" t="n">
+        <v>7521.59</v>
+      </c>
+      <c r="G50" s="45" t="n">
+        <v>0.001</v>
+      </c>
       <c r="H50" s="41" t="inlineStr">
         <is>
           <t>SELL</t>
@@ -7861,7 +8067,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A41"/>
+  <dimension ref="A1:A48"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.609375" defaultRowHeight="15"/>
   <cols>
     <col width="89.99609375" customWidth="1" style="37" min="1" max="1"/>
@@ -8068,7 +8274,6 @@
         </is>
       </c>
     </row>
-    <row r="33"/>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
@@ -8122,6 +8327,42 @@
       <c r="A41" t="inlineStr">
         <is>
           <t>- Blue-filled rows = added in the Jul 21 finalization pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>MA / MTD% methodology (added 2026-07-21):</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>- 5-Day / 7-Day MA after May 5 = average of the trailing 5/7 LOGGED closes (series has source gaps; not strictly consecutive trading days).</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>- MTD% baselines: Apr vs Mar 31 (6,528.52); May vs Apr 30 (7,155); Jun vs May 28 (7,599.96 - last logged May close, May 29 close unpublished); Jul vs Jun 30 (7,449.36).</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>- MA/MTD left blank on rows without a numeric close (Jul 16, Jul 20, holidays, PENDING).</t>
+        </is>
+      </c>
+    </row>
+    <row r="47"/>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>- MA/MTD% values computed at finalization (static values; environment could not run a live recalc engine).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tracker: fill all blank cells (oil spread/Δ/MTD/YoY, sector metrics, master log n/d flags)
Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HoDVqecVBj9mDnoNFdjBsS
</commit_message>
<xml_diff>
--- a/MI_PE_Tracking_System.xlsx
+++ b/MI_PE_Tracking_System.xlsx
@@ -1409,10 +1409,26 @@
       <c r="C18" s="20" t="n">
         <v>0.0146</v>
       </c>
-      <c r="D18" s="20" t="n"/>
-      <c r="E18" s="20" t="n"/>
-      <c r="F18" s="20" t="n"/>
-      <c r="G18" s="20" t="n"/>
+      <c r="D18" s="20" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E18" s="20" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="F18" s="20" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G18" s="20" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="H18" s="20" t="inlineStr">
         <is>
           <t>Tech steady</t>
@@ -1458,11 +1474,31 @@
       <c r="B19" s="20" t="n">
         <v>7412</v>
       </c>
-      <c r="C19" s="20" t="n"/>
-      <c r="D19" s="20" t="n"/>
-      <c r="E19" s="20" t="n"/>
-      <c r="F19" s="20" t="n"/>
-      <c r="G19" s="20" t="n"/>
+      <c r="C19" s="20" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="D19" s="20" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E19" s="20" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="F19" s="20" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G19" s="20" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="H19" s="20" t="inlineStr">
         <is>
           <t>AI leadership continues</t>
@@ -1508,11 +1544,31 @@
       <c r="B20" s="20" t="n">
         <v>7501.39</v>
       </c>
-      <c r="C20" s="20" t="n"/>
-      <c r="D20" s="20" t="n"/>
-      <c r="E20" s="20" t="n"/>
-      <c r="F20" s="20" t="n"/>
-      <c r="G20" s="20" t="n"/>
+      <c r="C20" s="20" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="D20" s="20" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E20" s="20" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="F20" s="20" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G20" s="20" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="H20" s="20" t="inlineStr">
         <is>
           <t>Chip/AI strength</t>
@@ -1560,15 +1616,31 @@
           <t>CLOSED</t>
         </is>
       </c>
-      <c r="C21" s="40" t="n"/>
+      <c r="C21" s="40" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="D21" s="40" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
       </c>
-      <c r="E21" s="40" t="n"/>
-      <c r="F21" s="40" t="n"/>
-      <c r="G21" s="40" t="n"/>
+      <c r="E21" s="40" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F21" s="40" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G21" s="40" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="H21" s="40" t="inlineStr">
         <is>
           <t>—</t>
@@ -1611,12 +1683,36 @@
           <t>May 27 2026</t>
         </is>
       </c>
-      <c r="B22" s="20" t="n"/>
-      <c r="C22" s="20" t="n"/>
-      <c r="D22" s="20" t="n"/>
-      <c r="E22" s="20" t="n"/>
-      <c r="F22" s="20" t="n"/>
-      <c r="G22" s="20" t="n"/>
+      <c r="B22" s="20" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="C22" s="20" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="D22" s="20" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E22" s="20" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="F22" s="20" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G22" s="20" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="H22" s="20" t="inlineStr">
         <is>
           <t>Micron joins $1T market-cap club</t>
@@ -1665,10 +1761,26 @@
       <c r="C23" s="20" t="n">
         <v>0.0026</v>
       </c>
-      <c r="D23" s="20" t="n"/>
-      <c r="E23" s="20" t="n"/>
-      <c r="F23" s="20" t="n"/>
-      <c r="G23" s="20" t="n"/>
+      <c r="D23" s="20" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E23" s="20" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="F23" s="20" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G23" s="20" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="H23" s="20" t="inlineStr">
         <is>
           <t>AI rally broadens</t>
@@ -1711,14 +1823,34 @@
           <t>May 29 2026</t>
         </is>
       </c>
-      <c r="B24" s="20" t="n"/>
-      <c r="C24" s="20" t="n"/>
+      <c r="B24" s="20" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="C24" s="20" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="D24" s="20" t="n">
         <v>26972.62</v>
       </c>
-      <c r="E24" s="20" t="n"/>
-      <c r="F24" s="20" t="n"/>
-      <c r="G24" s="20" t="n"/>
+      <c r="E24" s="20" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="F24" s="20" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G24" s="20" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="H24" s="20" t="inlineStr">
         <is>
           <t>Nasdaq intraday high 26,972.62</t>
@@ -1761,12 +1893,36 @@
           <t>Jun 1 2026</t>
         </is>
       </c>
-      <c r="B25" s="20" t="n"/>
-      <c r="C25" s="20" t="n"/>
-      <c r="D25" s="20" t="n"/>
-      <c r="E25" s="20" t="n"/>
-      <c r="F25" s="20" t="n"/>
-      <c r="G25" s="20" t="n"/>
+      <c r="B25" s="20" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="C25" s="20" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="D25" s="20" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E25" s="20" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="F25" s="20" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G25" s="20" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="H25" s="20" t="inlineStr">
         <is>
           <t>Tech rally overpowers oil spike</t>
@@ -1815,10 +1971,26 @@
       <c r="C26" s="21" t="n">
         <v>0.0013</v>
       </c>
-      <c r="D26" s="21" t="n"/>
-      <c r="E26" s="21" t="n"/>
-      <c r="F26" s="21" t="n"/>
-      <c r="G26" s="21" t="n"/>
+      <c r="D26" s="21" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E26" s="21" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="F26" s="21" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G26" s="21" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="H26" s="21" t="inlineStr">
         <is>
           <t>AI/chip melt-up</t>
@@ -1864,11 +2036,31 @@
       <c r="B27" s="40" t="n">
         <v>7583.95</v>
       </c>
-      <c r="C27" s="40" t="n"/>
-      <c r="D27" s="40" t="n"/>
-      <c r="E27" s="40" t="n"/>
-      <c r="F27" s="40" t="n"/>
-      <c r="G27" s="40" t="n"/>
+      <c r="C27" s="40" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="D27" s="40" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E27" s="40" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="F27" s="40" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G27" s="40" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="H27" s="40" t="inlineStr">
         <is>
           <t>Near-record into chip rout</t>
@@ -1917,8 +2109,16 @@
       <c r="C28" s="21" t="n">
         <v>-0.0264</v>
       </c>
-      <c r="D28" s="21" t="n"/>
-      <c r="E28" s="21" t="n"/>
+      <c r="D28" s="21" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E28" s="21" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="F28" s="21" t="n">
         <v>93.45</v>
       </c>
@@ -1973,10 +2173,26 @@
       <c r="C29" s="40" t="n">
         <v>0.003</v>
       </c>
-      <c r="D29" s="40" t="n"/>
-      <c r="E29" s="40" t="n"/>
-      <c r="F29" s="40" t="n"/>
-      <c r="G29" s="40" t="n"/>
+      <c r="D29" s="40" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E29" s="40" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="F29" s="40" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G29" s="40" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="H29" s="40" t="inlineStr">
         <is>
           <t>Chip rebound fails to hold</t>
@@ -2025,10 +2241,26 @@
       <c r="C30" s="40" t="n">
         <v>-0.0026</v>
       </c>
-      <c r="D30" s="40" t="n"/>
-      <c r="E30" s="40" t="n"/>
-      <c r="F30" s="40" t="n"/>
-      <c r="G30" s="40" t="n"/>
+      <c r="D30" s="40" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E30" s="40" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="F30" s="40" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G30" s="40" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="H30" s="40" t="inlineStr">
         <is>
           <t>Chip surge loses momentum</t>
@@ -2077,10 +2309,26 @@
       <c r="C31" s="40" t="n">
         <v>-0.0162</v>
       </c>
-      <c r="D31" s="40" t="n"/>
-      <c r="E31" s="40" t="n"/>
-      <c r="F31" s="40" t="n"/>
-      <c r="G31" s="40" t="n"/>
+      <c r="D31" s="40" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E31" s="40" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="F31" s="40" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G31" s="40" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="H31" s="40" t="inlineStr">
         <is>
           <t>Selloff deepens</t>
@@ -2129,10 +2377,26 @@
       <c r="C32" s="40" t="n">
         <v>0.0175</v>
       </c>
-      <c r="D32" s="40" t="n"/>
-      <c r="E32" s="40" t="n"/>
-      <c r="F32" s="40" t="n"/>
-      <c r="G32" s="40" t="n"/>
+      <c r="D32" s="40" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E32" s="40" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="F32" s="40" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G32" s="40" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="H32" s="40" t="inlineStr">
         <is>
           <t>Sharp rebound</t>
@@ -2181,10 +2445,26 @@
       <c r="C33" s="40" t="n">
         <v>0.005</v>
       </c>
-      <c r="D33" s="40" t="n"/>
-      <c r="E33" s="40" t="n"/>
-      <c r="F33" s="40" t="n"/>
-      <c r="G33" s="40" t="n"/>
+      <c r="D33" s="40" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E33" s="40" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="F33" s="40" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G33" s="40" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="H33" s="40" t="inlineStr">
         <is>
           <t>Recovery extends</t>
@@ -2233,10 +2513,26 @@
       <c r="C34" s="40" t="n">
         <v>0.0165</v>
       </c>
-      <c r="D34" s="40" t="n"/>
-      <c r="E34" s="40" t="n"/>
-      <c r="F34" s="40" t="n"/>
-      <c r="G34" s="40" t="n"/>
+      <c r="D34" s="40" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E34" s="40" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="F34" s="40" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G34" s="40" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="H34" s="40" t="inlineStr">
         <is>
           <t>SpaceX rally extends</t>
@@ -2285,10 +2581,26 @@
       <c r="C35" s="40" t="n">
         <v>-0.0057</v>
       </c>
-      <c r="D35" s="40" t="n"/>
-      <c r="E35" s="40" t="n"/>
-      <c r="F35" s="40" t="n"/>
-      <c r="G35" s="40" t="n"/>
+      <c r="D35" s="40" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E35" s="40" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="F35" s="40" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G35" s="40" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="H35" s="40" t="inlineStr">
         <is>
           <t>Warsh first-meeting jitters</t>
@@ -2343,8 +2655,16 @@
       <c r="E36" s="21" t="n">
         <v>-0.0134</v>
       </c>
-      <c r="F36" s="21" t="n"/>
-      <c r="G36" s="21" t="n"/>
+      <c r="F36" s="21" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G36" s="21" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="H36" s="21" t="inlineStr">
         <is>
           <t>Chips slide into Fed day</t>
@@ -2399,8 +2719,16 @@
       <c r="E37" s="21" t="n">
         <v>0.015</v>
       </c>
-      <c r="F37" s="21" t="n"/>
-      <c r="G37" s="21" t="n"/>
+      <c r="F37" s="21" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G37" s="21" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="H37" s="21" t="inlineStr">
         <is>
           <t>Chips fuel comeback</t>
@@ -2448,15 +2776,31 @@
           <t>CLOSED</t>
         </is>
       </c>
-      <c r="C38" s="21" t="n"/>
+      <c r="C38" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="D38" s="21" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
       </c>
-      <c r="E38" s="21" t="n"/>
-      <c r="F38" s="21" t="n"/>
-      <c r="G38" s="21" t="n"/>
+      <c r="E38" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F38" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G38" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="H38" s="21" t="inlineStr">
         <is>
           <t>—</t>
@@ -2499,10 +2843,26 @@
           <t>Jun 20 2026</t>
         </is>
       </c>
-      <c r="B39" s="21" t="n"/>
-      <c r="C39" s="21" t="n"/>
-      <c r="D39" s="21" t="n"/>
-      <c r="E39" s="21" t="n"/>
+      <c r="B39" s="21" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="C39" s="21" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="D39" s="21" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E39" s="21" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="F39" s="21" t="n">
         <v>77.54000000000001</v>
       </c>
@@ -2683,6 +3043,16 @@
       <c r="E42" t="n">
         <v>-0.0043</v>
       </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="H42" t="inlineStr">
         <is>
           <t>Chips slide ahead of Micron</t>
@@ -2737,6 +3107,16 @@
       <c r="E43" t="n">
         <v>-0.0046</v>
       </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="H43" t="inlineStr">
         <is>
           <t>Tech soft</t>
@@ -2779,9 +3159,34 @@
           <t>Jun 26 2026</t>
         </is>
       </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="F44" t="n">
         <v>69.5</v>
       </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="H44" t="inlineStr">
         <is>
           <t>Tread water amid tech sell-off</t>
@@ -2830,9 +3235,19 @@
       <c r="C45" t="n">
         <v>0.012</v>
       </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="E45" t="n">
         <v>0.02</v>
       </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="G45" t="n">
         <v>73.17</v>
       </c>
@@ -2890,6 +3305,16 @@
       <c r="E46" t="n">
         <v>0.0029</v>
       </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="H46" t="inlineStr">
         <is>
           <t>Nasdaq +0.29%</t>
@@ -2938,6 +3363,16 @@
       <c r="C47" t="n">
         <v>0.0045</v>
       </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="F47" t="n">
         <v>68.58</v>
       </c>
@@ -2992,9 +3427,17 @@
       <c r="C48" t="n">
         <v>-0.0039</v>
       </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="E48" t="n">
         <v>-0.0118</v>
       </c>
+      <c r="F48" t="n">
+        <v>68</v>
+      </c>
       <c r="G48" t="n">
         <v>68</v>
       </c>
@@ -3045,15 +3488,31 @@
           <t>CLOSED</t>
         </is>
       </c>
-      <c r="C49" s="41" t="n"/>
+      <c r="C49" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="D49" s="41" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
       </c>
-      <c r="E49" s="41" t="n"/>
-      <c r="F49" s="41" t="n"/>
-      <c r="G49" s="41" t="n"/>
+      <c r="E49" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F49" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G49" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="H49" s="41" t="inlineStr">
         <is>
           <t>—</t>
@@ -3108,8 +3567,16 @@
       <c r="E50" s="41" t="n">
         <v>0.0112</v>
       </c>
-      <c r="F50" s="41" t="n"/>
-      <c r="G50" s="41" t="n"/>
+      <c r="F50" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G50" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="H50" s="41" t="inlineStr">
         <is>
           <t>AI optimism revives</t>
@@ -3164,8 +3631,16 @@
       <c r="E51" s="41" t="n">
         <v>-0.0116</v>
       </c>
-      <c r="F51" s="41" t="n"/>
-      <c r="G51" s="41" t="n"/>
+      <c r="F51" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G51" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="H51" s="41" t="inlineStr">
         <is>
           <t>Tech gives back</t>
@@ -3214,8 +3689,16 @@
       <c r="C52" s="41" t="n">
         <v>-0.0028</v>
       </c>
-      <c r="D52" s="41" t="n"/>
-      <c r="E52" s="41" t="n"/>
+      <c r="D52" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E52" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="F52" s="41" t="n">
         <v>73.52</v>
       </c>
@@ -3270,10 +3753,26 @@
       <c r="C53" s="41" t="n">
         <v>0.0081</v>
       </c>
-      <c r="D53" s="41" t="n"/>
-      <c r="E53" s="41" t="n"/>
-      <c r="F53" s="41" t="n"/>
-      <c r="G53" s="41" t="n"/>
+      <c r="D53" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E53" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="F53" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G53" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="H53" s="41" t="inlineStr">
         <is>
           <t>Semis jump</t>
@@ -3328,8 +3827,16 @@
       <c r="E54" s="41" t="n">
         <v>0.0029</v>
       </c>
-      <c r="F54" s="41" t="n"/>
-      <c r="G54" s="41" t="n"/>
+      <c r="F54" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G54" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="H54" s="41" t="inlineStr">
         <is>
           <t>Tech-led winning week</t>
@@ -3378,10 +3885,26 @@
       <c r="C55" s="41" t="n">
         <v>-0.008</v>
       </c>
-      <c r="D55" s="41" t="n"/>
-      <c r="E55" s="41" t="n"/>
-      <c r="F55" s="41" t="n"/>
-      <c r="G55" s="41" t="n"/>
+      <c r="D55" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E55" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="F55" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G55" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="H55" s="41" t="inlineStr">
         <is>
           <t>Drift lower</t>
@@ -3436,8 +3959,16 @@
       <c r="E56" s="41" t="n">
         <v>0.008999999999999999</v>
       </c>
-      <c r="F56" s="41" t="n"/>
-      <c r="G56" s="41" t="n"/>
+      <c r="F56" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G56" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="H56" s="41" t="inlineStr">
         <is>
           <t>Nasdaq +0.9%</t>
@@ -3492,8 +4023,16 @@
       <c r="E57" s="41" t="n">
         <v>-0.0147</v>
       </c>
-      <c r="F57" s="41" t="n"/>
-      <c r="G57" s="41" t="n"/>
+      <c r="F57" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G57" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="H57" s="41" t="inlineStr">
         <is>
           <t>Alphabet &amp; chips sell off; SpaceX below IPO price</t>
@@ -3536,16 +4075,32 @@
           <t>Jul 16 2026</t>
         </is>
       </c>
-      <c r="B58" s="41" t="n"/>
+      <c r="B58" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="C58" s="41" t="n">
         <v>-0.0037</v>
       </c>
-      <c r="D58" s="41" t="n"/>
+      <c r="D58" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="E58" s="41" t="n">
         <v>-0.0076</v>
       </c>
-      <c r="F58" s="41" t="n"/>
-      <c r="G58" s="41" t="n"/>
+      <c r="F58" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G58" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="H58" s="41" t="inlineStr">
         <is>
           <t>Semiconductor slide continues</t>
@@ -3600,8 +4155,16 @@
       <c r="E59" s="41" t="n">
         <v>-0.014</v>
       </c>
-      <c r="F59" s="41" t="n"/>
-      <c r="G59" s="41" t="n"/>
+      <c r="F59" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G59" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="H59" s="41" t="inlineStr">
         <is>
           <t>MOONSHOT AI SHOCK: Chinese startup rivals US models; global tech rout</t>
@@ -3644,11 +4207,31 @@
           <t>Jul 20 2026</t>
         </is>
       </c>
-      <c r="B60" s="41" t="n"/>
-      <c r="C60" s="41" t="n"/>
-      <c r="D60" s="41" t="n"/>
-      <c r="E60" s="41" t="n"/>
-      <c r="F60" s="41" t="n"/>
+      <c r="B60" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="C60" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="D60" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E60" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="F60" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="G60" s="41" t="n">
         <v>90</v>
       </c>
@@ -3699,15 +4282,31 @@
           <t>PENDING</t>
         </is>
       </c>
-      <c r="C61" s="41" t="n"/>
+      <c r="C61" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="D61" s="41" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
       </c>
-      <c r="E61" s="41" t="n"/>
-      <c r="F61" s="41" t="n"/>
-      <c r="G61" s="41" t="n"/>
+      <c r="E61" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F61" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G61" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="H61" s="41" t="inlineStr">
         <is>
           <t>—</t>
@@ -3860,9 +4459,8 @@
       <c r="F5" s="5" t="n">
         <v>7109.14</v>
       </c>
-      <c r="G5" s="6">
-        <f>(B5-6528.52)/6528.52</f>
-        <v/>
+      <c r="G5" s="6" t="n">
+        <v>0.08890000000000001</v>
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
@@ -3889,13 +4487,11 @@
       <c r="B6" s="5" t="n">
         <v>7064.01</v>
       </c>
-      <c r="C6" s="5">
-        <f>B6-B5</f>
-        <v/>
-      </c>
-      <c r="D6" s="6">
-        <f>(B6-B5)/B5</f>
-        <v/>
+      <c r="C6" s="5" t="n">
+        <v>-45.13</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>-0.0063</v>
       </c>
       <c r="E6" s="5" t="n">
         <v>7086.58</v>
@@ -3903,9 +4499,8 @@
       <c r="F6" s="5" t="n">
         <v>7086.58</v>
       </c>
-      <c r="G6" s="6">
-        <f>(B6-6528.52)/6528.52</f>
-        <v/>
+      <c r="G6" s="6" t="n">
+        <v>0.082</v>
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
@@ -3932,13 +4527,11 @@
       <c r="B7" s="5" t="n">
         <v>7137.9</v>
       </c>
-      <c r="C7" s="5">
-        <f>B7-B6</f>
-        <v/>
-      </c>
-      <c r="D7" s="6">
-        <f>(B7-B6)/B6</f>
-        <v/>
+      <c r="C7" s="5" t="n">
+        <v>73.89</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>0.0105</v>
       </c>
       <c r="E7" s="5" t="n">
         <v>7123.52</v>
@@ -3946,9 +4539,8 @@
       <c r="F7" s="5" t="n">
         <v>7123.52</v>
       </c>
-      <c r="G7" s="6">
-        <f>(B7-6528.52)/6528.52</f>
-        <v/>
+      <c r="G7" s="6" t="n">
+        <v>0.09329999999999999</v>
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
@@ -3975,13 +4567,11 @@
       <c r="B8" s="5" t="n">
         <v>7108.4</v>
       </c>
-      <c r="C8" s="5">
-        <f>B8-B7</f>
-        <v/>
-      </c>
-      <c r="D8" s="6">
-        <f>(B8-B7)/B7</f>
-        <v/>
+      <c r="C8" s="5" t="n">
+        <v>-29.5</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>-0.0041</v>
       </c>
       <c r="E8" s="5" t="n">
         <v>7108.77</v>
@@ -3989,9 +4579,8 @@
       <c r="F8" s="5" t="n">
         <v>7108.77</v>
       </c>
-      <c r="G8" s="6">
-        <f>(B8-6528.52)/6528.52</f>
-        <v/>
+      <c r="G8" s="6" t="n">
+        <v>0.0888</v>
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
@@ -4018,13 +4607,11 @@
       <c r="B9" s="5" t="n">
         <v>7165.08</v>
       </c>
-      <c r="C9" s="5">
-        <f>B9-B8</f>
-        <v/>
-      </c>
-      <c r="D9" s="6">
-        <f>(B9-B8)/B8</f>
-        <v/>
+      <c r="C9" s="5" t="n">
+        <v>56.68</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>0.008</v>
       </c>
       <c r="E9" s="5" t="n">
         <v>7137.11</v>
@@ -4032,9 +4619,8 @@
       <c r="F9" s="5" t="n">
         <v>7137.11</v>
       </c>
-      <c r="G9" s="6">
-        <f>(B9-6528.52)/6528.52</f>
-        <v/>
+      <c r="G9" s="6" t="n">
+        <v>0.0975</v>
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
@@ -4061,13 +4647,11 @@
       <c r="B10" s="10" t="n">
         <v>7138.8</v>
       </c>
-      <c r="C10" s="10">
-        <f>B10-B9</f>
-        <v/>
-      </c>
-      <c r="D10" s="11">
-        <f>(B10-B9)/B9</f>
-        <v/>
+      <c r="C10" s="10" t="n">
+        <v>-26.28</v>
+      </c>
+      <c r="D10" s="11" t="n">
+        <v>-0.0037</v>
       </c>
       <c r="E10" s="10" t="n">
         <v>7101.41</v>
@@ -4075,9 +4659,8 @@
       <c r="F10" s="10" t="n">
         <v>7123.97</v>
       </c>
-      <c r="G10" s="11">
-        <f>(B10-6528.52)/6528.52</f>
-        <v/>
+      <c r="G10" s="11" t="n">
+        <v>0.0935</v>
       </c>
       <c r="H10" s="12" t="inlineStr">
         <is>
@@ -4104,13 +4687,11 @@
       <c r="B11" s="10" t="n">
         <v>7173.91</v>
       </c>
-      <c r="C11" s="10">
-        <f>B11-B10</f>
-        <v/>
-      </c>
-      <c r="D11" s="11">
-        <f>(B11-B10)/B10</f>
-        <v/>
+      <c r="C11" s="10" t="n">
+        <v>35.11</v>
+      </c>
+      <c r="D11" s="11" t="n">
+        <v>0.0049</v>
       </c>
       <c r="E11" s="10" t="n">
         <v>7155.9</v>
@@ -4118,9 +4699,8 @@
       <c r="F11" s="10" t="n">
         <v>7141.52</v>
       </c>
-      <c r="G11" s="11">
-        <f>(B11-6528.52)/6528.52</f>
-        <v/>
+      <c r="G11" s="11" t="n">
+        <v>0.0989</v>
       </c>
       <c r="H11" s="12" t="inlineStr">
         <is>
@@ -4147,13 +4727,11 @@
       <c r="B12" s="10" t="n">
         <v>7135.95</v>
       </c>
-      <c r="C12" s="10">
-        <f>B12-B11</f>
-        <v/>
-      </c>
-      <c r="D12" s="11">
-        <f>(B12-B11)/B11</f>
-        <v/>
+      <c r="C12" s="10" t="n">
+        <v>-37.96</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>-0.0053</v>
       </c>
       <c r="E12" s="10" t="n">
         <v>7122.17</v>
@@ -4161,9 +4739,8 @@
       <c r="F12" s="10" t="n">
         <v>7099.98</v>
       </c>
-      <c r="G12" s="11">
-        <f>(B12-6528.52)/6528.52</f>
-        <v/>
+      <c r="G12" s="11" t="n">
+        <v>0.093</v>
       </c>
       <c r="H12" s="12" t="inlineStr">
         <is>
@@ -4190,13 +4767,11 @@
       <c r="B13" s="10" t="n">
         <v>7155</v>
       </c>
-      <c r="C13" s="10">
-        <f>B13-B12</f>
-        <v/>
-      </c>
-      <c r="D13" s="11">
-        <f>(B13-B12)/B12</f>
-        <v/>
+      <c r="C13" s="10" t="n">
+        <v>19.05</v>
+      </c>
+      <c r="D13" s="11" t="n">
+        <v>0.0027</v>
       </c>
       <c r="E13" s="10" t="n">
         <v>7160.04</v>
@@ -4204,9 +4779,8 @@
       <c r="F13" s="10" t="n">
         <v>7146.45</v>
       </c>
-      <c r="G13" s="11">
-        <f>(B13-6528.52)/6528.52</f>
-        <v/>
+      <c r="G13" s="11" t="n">
+        <v>0.096</v>
       </c>
       <c r="H13" s="12" t="inlineStr">
         <is>
@@ -4233,13 +4807,11 @@
       <c r="B14" s="10" t="n">
         <v>7230.12</v>
       </c>
-      <c r="C14" s="10">
-        <f>B14-B13</f>
-        <v/>
-      </c>
-      <c r="D14" s="11">
-        <f>(B14-B13)/B13</f>
-        <v/>
+      <c r="C14" s="10" t="n">
+        <v>75.12</v>
+      </c>
+      <c r="D14" s="11" t="n">
+        <v>0.0105</v>
       </c>
       <c r="E14" s="10" t="n">
         <v>7184.46</v>
@@ -4247,9 +4819,8 @@
       <c r="F14" s="10" t="n">
         <v>7169.26</v>
       </c>
-      <c r="G14" s="11">
-        <f>(B14-6528.52)/6528.52</f>
-        <v/>
+      <c r="G14" s="11" t="n">
+        <v>0.1075</v>
       </c>
       <c r="H14" s="12" t="inlineStr">
         <is>
@@ -4276,13 +4847,11 @@
       <c r="B15" s="10" t="n">
         <v>7200.75</v>
       </c>
-      <c r="C15" s="10">
-        <f>B15-B14</f>
-        <v/>
-      </c>
-      <c r="D15" s="11">
-        <f>(B15-B14)/B14</f>
-        <v/>
+      <c r="C15" s="10" t="n">
+        <v>-29.37</v>
+      </c>
+      <c r="D15" s="11" t="n">
+        <v>-0.0041</v>
       </c>
       <c r="E15" s="10" t="n">
         <v>7187.33</v>
@@ -4290,9 +4859,8 @@
       <c r="F15" s="10" t="n">
         <v>7182.91</v>
       </c>
-      <c r="G15" s="11">
-        <f>(B15-6528.52)/6528.52</f>
-        <v/>
+      <c r="G15" s="11" t="n">
+        <v>0.103</v>
       </c>
       <c r="H15" s="12" t="inlineStr">
         <is>
@@ -4319,13 +4887,11 @@
       <c r="B16" s="10" t="n">
         <v>7259.22</v>
       </c>
-      <c r="C16" s="10">
-        <f>B16-B15</f>
-        <v/>
-      </c>
-      <c r="D16" s="11">
-        <f>(B16-B15)/B15</f>
-        <v/>
+      <c r="C16" s="10" t="n">
+        <v>58.47</v>
+      </c>
+      <c r="D16" s="11" t="n">
+        <v>0.0081</v>
       </c>
       <c r="E16" s="10" t="n">
         <v>7197.59</v>
@@ -4333,9 +4899,8 @@
       <c r="F16" s="10" t="n">
         <v>7199.01</v>
       </c>
-      <c r="G16" s="11">
-        <f>(B16-6528.52)/6528.52</f>
-        <v/>
+      <c r="G16" s="11" t="n">
+        <v>0.1119</v>
       </c>
       <c r="H16" s="12" t="inlineStr">
         <is>
@@ -4362,7 +4927,9 @@
       <c r="B17" s="18" t="n">
         <v>7365.12</v>
       </c>
-      <c r="C17" s="18" t="n"/>
+      <c r="C17" s="18" t="n">
+        <v>105.9</v>
+      </c>
       <c r="D17" s="18" t="n">
         <v>0.0146</v>
       </c>
@@ -4400,8 +4967,12 @@
       <c r="B18" s="18" t="n">
         <v>7412</v>
       </c>
-      <c r="C18" s="18" t="n"/>
-      <c r="D18" s="18" t="n"/>
+      <c r="C18" s="18" t="n">
+        <v>46.88</v>
+      </c>
+      <c r="D18" s="43" t="n">
+        <v>0.0064</v>
+      </c>
       <c r="E18" s="42" t="n">
         <v>7293.44</v>
       </c>
@@ -4436,8 +5007,12 @@
       <c r="B19" s="18" t="n">
         <v>7501.39</v>
       </c>
-      <c r="C19" s="18" t="n"/>
-      <c r="D19" s="18" t="n"/>
+      <c r="C19" s="18" t="n">
+        <v>89.39</v>
+      </c>
+      <c r="D19" s="43" t="n">
+        <v>0.0121</v>
+      </c>
       <c r="E19" s="42" t="n">
         <v>7347.7</v>
       </c>
@@ -4472,7 +5047,9 @@
       <c r="B20" s="18" t="n">
         <v>7599.96</v>
       </c>
-      <c r="C20" s="18" t="n"/>
+      <c r="C20" s="18" t="n">
+        <v>98.56999999999999</v>
+      </c>
       <c r="D20" s="18" t="n">
         <v>0.0026</v>
       </c>
@@ -4510,7 +5087,9 @@
       <c r="B21" s="18" t="n">
         <v>7609.78</v>
       </c>
-      <c r="C21" s="18" t="n"/>
+      <c r="C21" s="18" t="n">
+        <v>9.82</v>
+      </c>
       <c r="D21" s="18" t="n">
         <v>0.0013</v>
       </c>
@@ -4548,8 +5127,12 @@
       <c r="B22" s="41" t="n">
         <v>7583.95</v>
       </c>
-      <c r="C22" s="41" t="n"/>
-      <c r="D22" s="41" t="n"/>
+      <c r="C22" s="41" t="n">
+        <v>-25.83</v>
+      </c>
+      <c r="D22" s="45" t="n">
+        <v>-0.0034</v>
+      </c>
       <c r="E22" s="44" t="n">
         <v>7541.42</v>
       </c>
@@ -4584,7 +5167,9 @@
       <c r="B23" s="19" t="n">
         <v>7383.74</v>
       </c>
-      <c r="C23" s="19" t="n"/>
+      <c r="C23" s="19" t="n">
+        <v>-200.21</v>
+      </c>
       <c r="D23" s="19" t="n">
         <v>-0.0264</v>
       </c>
@@ -4902,7 +5487,9 @@
       <c r="B31" s="19" t="n">
         <v>7420.1</v>
       </c>
-      <c r="C31" s="19" t="n"/>
+      <c r="C31" s="19" t="n">
+        <v>-90.88</v>
+      </c>
       <c r="D31" s="19" t="n">
         <v>-0.0121</v>
       </c>
@@ -5140,6 +5727,9 @@
       <c r="B37" t="n">
         <v>7445</v>
       </c>
+      <c r="C37" t="n">
+        <v>87.51000000000001</v>
+      </c>
       <c r="D37" t="n">
         <v>0.012</v>
       </c>
@@ -5217,6 +5807,9 @@
       <c r="B39" t="n">
         <v>7483</v>
       </c>
+      <c r="C39" t="n">
+        <v>33.64</v>
+      </c>
       <c r="D39" t="n">
         <v>0.0045</v>
       </c>
@@ -5254,6 +5847,9 @@
       <c r="B40" t="n">
         <v>7453.96</v>
       </c>
+      <c r="C40" t="n">
+        <v>-29.04</v>
+      </c>
       <c r="D40" t="n">
         <v>-0.0039</v>
       </c>
@@ -5291,7 +5887,9 @@
       <c r="B41" s="41" t="n">
         <v>7537.43</v>
       </c>
-      <c r="C41" s="41" t="n"/>
+      <c r="C41" s="41" t="n">
+        <v>83.47</v>
+      </c>
       <c r="D41" s="41" t="n">
         <v>0.0072</v>
       </c>
@@ -5606,14 +6204,34 @@
           <t>Jul 16</t>
         </is>
       </c>
-      <c r="B49" s="41" t="n"/>
-      <c r="C49" s="41" t="n"/>
+      <c r="B49" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="C49" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="D49" s="41" t="n">
         <v>-0.0037</v>
       </c>
-      <c r="E49" s="41" t="n"/>
-      <c r="F49" s="41" t="n"/>
-      <c r="G49" s="41" t="n"/>
+      <c r="E49" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="F49" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G49" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="H49" s="41" t="inlineStr">
         <is>
           <t>SELL</t>
@@ -5639,7 +6257,9 @@
       <c r="B50" s="41" t="n">
         <v>7457</v>
       </c>
-      <c r="C50" s="41" t="n"/>
+      <c r="C50" s="41" t="n">
+        <v>-76.77</v>
+      </c>
       <c r="D50" s="41" t="n">
         <v>-0.0102</v>
       </c>
@@ -5674,12 +6294,36 @@
           <t>Jul 20</t>
         </is>
       </c>
-      <c r="B51" s="41" t="n"/>
-      <c r="C51" s="41" t="n"/>
-      <c r="D51" s="41" t="n"/>
-      <c r="E51" s="41" t="n"/>
-      <c r="F51" s="41" t="n"/>
-      <c r="G51" s="41" t="n"/>
+      <c r="B51" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="C51" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="D51" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E51" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="F51" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G51" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="H51" s="41" t="inlineStr">
         <is>
           <t>SELL</t>
@@ -5707,11 +6351,31 @@
           <t>PENDING</t>
         </is>
       </c>
-      <c r="C52" s="41" t="n"/>
-      <c r="D52" s="41" t="n"/>
-      <c r="E52" s="41" t="n"/>
-      <c r="F52" s="41" t="n"/>
-      <c r="G52" s="41" t="n"/>
+      <c r="C52" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="D52" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E52" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="F52" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G52" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="H52" s="41" t="inlineStr">
         <is>
           <t>—</t>
@@ -5823,20 +6487,17 @@
       <c r="C5" s="14" t="n">
         <v>96.26000000000001</v>
       </c>
-      <c r="D5" s="14">
-        <f>C5-B5</f>
-        <v/>
+      <c r="D5" s="14" t="n">
+        <v>0</v>
       </c>
       <c r="E5" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="6">
-        <f>(C5-102)/102</f>
-        <v/>
-      </c>
-      <c r="G5" s="6">
-        <f>(C5-65.83)/65.83</f>
-        <v/>
+      <c r="F5" s="6" t="n">
+        <v>-0.0563</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>0.4623</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
@@ -5856,21 +6517,17 @@
       <c r="C6" s="14" t="n">
         <v>96.5</v>
       </c>
-      <c r="D6" s="14">
-        <f>C6-B6</f>
-        <v/>
-      </c>
-      <c r="E6" s="6">
-        <f>(B6-B5)/B5</f>
-        <v/>
-      </c>
-      <c r="F6" s="6">
-        <f>(C6-102)/102</f>
-        <v/>
-      </c>
-      <c r="G6" s="6">
-        <f>(C6-65.83)/65.83</f>
-        <v/>
+      <c r="D6" s="14" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>-0.0027</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>-0.0539</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>0.4659</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
@@ -5890,21 +6547,17 @@
       <c r="C7" s="14" t="n">
         <v>96</v>
       </c>
-      <c r="D7" s="14">
-        <f>C7-B7</f>
-        <v/>
-      </c>
-      <c r="E7" s="6">
-        <f>(B7-B6)/B6</f>
-        <v/>
-      </c>
-      <c r="F7" s="6">
-        <f>(C7-102)/102</f>
-        <v/>
-      </c>
-      <c r="G7" s="6">
-        <f>(C7-65.83)/65.83</f>
-        <v/>
+      <c r="D7" s="14" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>-0.0052</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>-0.0588</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>0.4583</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
@@ -5924,21 +6577,17 @@
       <c r="C8" s="14" t="n">
         <v>105.33</v>
       </c>
-      <c r="D8" s="14">
-        <f>C8-B8</f>
-        <v/>
-      </c>
-      <c r="E8" s="6">
-        <f>(B8-B7)/B7</f>
-        <v/>
-      </c>
-      <c r="F8" s="6">
-        <f>(C8-102)/102</f>
-        <v/>
-      </c>
-      <c r="G8" s="6">
-        <f>(C8-65.83)/65.83</f>
-        <v/>
+      <c r="D8" s="14" t="n">
+        <v>10.93</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>-0.0115</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>0.0326</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>0.6</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
@@ -5958,21 +6607,17 @@
       <c r="C9" s="14" t="n">
         <v>105.33</v>
       </c>
-      <c r="D9" s="14">
-        <f>C9-B9</f>
-        <v/>
-      </c>
-      <c r="E9" s="6">
-        <f>(B9-B8)/B8</f>
-        <v/>
-      </c>
-      <c r="F9" s="6">
-        <f>(C9-102)/102</f>
-        <v/>
-      </c>
-      <c r="G9" s="6">
-        <f>(C9-65.83)/65.83</f>
-        <v/>
+      <c r="D9" s="14" t="n">
+        <v>11.29</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>-0.0038</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>0.0326</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>0.6</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
@@ -5992,21 +6637,17 @@
       <c r="C10" s="14" t="n">
         <v>105.2</v>
       </c>
-      <c r="D10" s="14">
-        <f>C10-B10</f>
-        <v/>
-      </c>
-      <c r="E10" s="6">
-        <f>(B10-B9)/B9</f>
-        <v/>
-      </c>
-      <c r="F10" s="6">
-        <f>(C10-102)/102</f>
-        <v/>
-      </c>
-      <c r="G10" s="6">
-        <f>(C10-65.83)/65.83</f>
-        <v/>
+      <c r="D10" s="14" t="n">
+        <v>11.52</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>-0.0038</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>0.0314</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>0.5981</v>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
@@ -6026,21 +6667,17 @@
       <c r="C11" s="15" t="n">
         <v>107</v>
       </c>
-      <c r="D11" s="15">
-        <f>C11-B11</f>
-        <v/>
-      </c>
-      <c r="E11" s="11">
-        <f>(B11-B10)/B10</f>
-        <v/>
-      </c>
-      <c r="F11" s="11">
-        <f>(C11-102)/102</f>
-        <v/>
-      </c>
-      <c r="G11" s="11">
-        <f>(C11-65.83)/65.83</f>
-        <v/>
+      <c r="D11" s="15" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>0.0194</v>
+      </c>
+      <c r="F11" s="11" t="n">
+        <v>0.049</v>
+      </c>
+      <c r="G11" s="11" t="n">
+        <v>0.6254</v>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
@@ -6060,21 +6697,17 @@
       <c r="C12" s="15" t="n">
         <v>108</v>
       </c>
-      <c r="D12" s="15">
-        <f>C12-B12</f>
-        <v/>
-      </c>
-      <c r="E12" s="11">
-        <f>(B12-B11)/B11</f>
-        <v/>
-      </c>
-      <c r="F12" s="11">
-        <f>(C12-102)/102</f>
-        <v/>
-      </c>
-      <c r="G12" s="11">
-        <f>(C12-65.83)/65.83</f>
-        <v/>
+      <c r="D12" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>0.0052</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>0.0588</v>
+      </c>
+      <c r="G12" s="11" t="n">
+        <v>0.6405999999999999</v>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
@@ -6094,21 +6727,17 @@
       <c r="C13" s="15" t="n">
         <v>108.5</v>
       </c>
-      <c r="D13" s="15">
-        <f>C13-B13</f>
-        <v/>
-      </c>
-      <c r="E13" s="11">
-        <f>(B13-B12)/B12</f>
-        <v/>
-      </c>
-      <c r="F13" s="11">
-        <f>(C13-102)/102</f>
-        <v/>
-      </c>
-      <c r="G13" s="11">
-        <f>(C13-65.83)/65.83</f>
-        <v/>
+      <c r="D13" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="E13" s="11" t="n">
+        <v>0.0052</v>
+      </c>
+      <c r="F13" s="11" t="n">
+        <v>0.06370000000000001</v>
+      </c>
+      <c r="G13" s="11" t="n">
+        <v>0.6482</v>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
@@ -6128,21 +6757,17 @@
       <c r="C14" s="15" t="n">
         <v>107.8</v>
       </c>
-      <c r="D14" s="15">
-        <f>C14-B14</f>
-        <v/>
-      </c>
-      <c r="E14" s="11">
-        <f>(B14-B13)/B13</f>
-        <v/>
-      </c>
-      <c r="F14" s="11">
-        <f>(C14-102)/102</f>
-        <v/>
-      </c>
-      <c r="G14" s="11">
-        <f>(C14-65.83)/65.83</f>
-        <v/>
+      <c r="D14" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="E14" s="11" t="n">
+        <v>-0.0073</v>
+      </c>
+      <c r="F14" s="11" t="n">
+        <v>0.0569</v>
+      </c>
+      <c r="G14" s="11" t="n">
+        <v>0.6375999999999999</v>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
@@ -6162,21 +6787,17 @@
       <c r="C15" s="15" t="n">
         <v>107</v>
       </c>
-      <c r="D15" s="15">
-        <f>C15-B15</f>
-        <v/>
-      </c>
-      <c r="E15" s="11">
-        <f>(B15-B14)/B14</f>
-        <v/>
-      </c>
-      <c r="F15" s="11">
-        <f>(C15-102)/102</f>
-        <v/>
-      </c>
-      <c r="G15" s="11">
-        <f>(C15-65.83)/65.83</f>
-        <v/>
+      <c r="D15" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="E15" s="11" t="n">
+        <v>-0.008399999999999999</v>
+      </c>
+      <c r="F15" s="11" t="n">
+        <v>0.049</v>
+      </c>
+      <c r="G15" s="11" t="n">
+        <v>0.6254</v>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
@@ -6196,21 +6817,17 @@
       <c r="C16" s="15" t="n">
         <v>109.87</v>
       </c>
-      <c r="D16" s="15">
-        <f>C16-B16</f>
-        <v/>
-      </c>
-      <c r="E16" s="11">
-        <f>(B16-B15)/B15</f>
-        <v/>
-      </c>
-      <c r="F16" s="11">
-        <f>(C16-102)/102</f>
-        <v/>
-      </c>
-      <c r="G16" s="11">
-        <f>(C16-65.83)/65.83</f>
-        <v/>
+      <c r="D16" s="15" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="E16" s="11" t="n">
+        <v>0.0765</v>
+      </c>
+      <c r="F16" s="11" t="n">
+        <v>0.0772</v>
+      </c>
+      <c r="G16" s="11" t="n">
+        <v>0.669</v>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
@@ -6230,21 +6847,17 @@
       <c r="C17" s="15" t="n">
         <v>109.87</v>
       </c>
-      <c r="D17" s="15">
-        <f>C17-B17</f>
-        <v/>
-      </c>
-      <c r="E17" s="11">
-        <f>(B17-B16)/B16</f>
-        <v/>
-      </c>
-      <c r="F17" s="11">
-        <f>(C17-102)/102</f>
-        <v/>
-      </c>
-      <c r="G17" s="11">
-        <f>(C17-65.83)/65.83</f>
-        <v/>
+      <c r="D17" s="15" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="E17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="11" t="n">
+        <v>0.0772</v>
+      </c>
+      <c r="G17" s="11" t="n">
+        <v>0.669</v>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
@@ -6258,14 +6871,30 @@
           <t>May 15</t>
         </is>
       </c>
-      <c r="B18" s="18" t="n"/>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="C18" s="18" t="n">
         <v>113</v>
       </c>
-      <c r="D18" s="18" t="n"/>
-      <c r="E18" s="18" t="n"/>
-      <c r="F18" s="18" t="n"/>
-      <c r="G18" s="18" t="n"/>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E18" s="18" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="F18" s="43" t="n">
+        <v>0.0482</v>
+      </c>
+      <c r="G18" s="43" t="n">
+        <v>0.7165</v>
+      </c>
       <c r="H18" s="18" t="inlineStr">
         <is>
           <t>Brent peaks &gt;$113 on Hormuz disruption (2026 high)</t>
@@ -6287,9 +6916,15 @@
       <c r="D19" s="19" t="n">
         <v>3.99</v>
       </c>
-      <c r="E19" s="19" t="n"/>
-      <c r="F19" s="19" t="n"/>
-      <c r="G19" s="19" t="n"/>
+      <c r="E19" s="47" t="n">
+        <v>-0.0862</v>
+      </c>
+      <c r="F19" s="47" t="n">
+        <v>-0.1377</v>
+      </c>
+      <c r="G19" s="47" t="n">
+        <v>0.4802</v>
+      </c>
       <c r="H19" s="19" t="inlineStr">
         <is>
           <t>Post-gap; premium fading</t>
@@ -6311,9 +6946,15 @@
       <c r="D20" s="19" t="n">
         <v>3.03</v>
       </c>
-      <c r="E20" s="19" t="n"/>
-      <c r="F20" s="19" t="n"/>
-      <c r="G20" s="19" t="n"/>
+      <c r="E20" s="47" t="n">
+        <v>-0.1703</v>
+      </c>
+      <c r="F20" s="47" t="n">
+        <v>-0.287</v>
+      </c>
+      <c r="G20" s="47" t="n">
+        <v>0.2239</v>
+      </c>
       <c r="H20" s="19" t="inlineStr">
         <is>
           <t>Iran re-closed Hormuz; ceasefire tentative</t>
@@ -6335,9 +6976,15 @@
       <c r="D21" s="19" t="n">
         <v>4.11</v>
       </c>
-      <c r="E21" s="19" t="n"/>
-      <c r="F21" s="19" t="n"/>
-      <c r="G21" s="19" t="n"/>
+      <c r="E21" s="47" t="n">
+        <v>-0.0418</v>
+      </c>
+      <c r="F21" s="47" t="n">
+        <v>-0.3061</v>
+      </c>
+      <c r="G21" s="47" t="n">
+        <v>0.1911</v>
+      </c>
       <c r="H21" s="19" t="inlineStr">
         <is>
           <t>VP Vance 'good foundation'</t>
@@ -6359,9 +7006,15 @@
       <c r="D22" s="19" t="n">
         <v>4.6</v>
       </c>
-      <c r="E22" s="19" t="n"/>
-      <c r="F22" s="19" t="n"/>
-      <c r="G22" s="19" t="n"/>
+      <c r="E22" s="47" t="n">
+        <v>-0.0121</v>
+      </c>
+      <c r="F22" s="47" t="n">
+        <v>-0.3097</v>
+      </c>
+      <c r="G22" s="47" t="n">
+        <v>0.1849</v>
+      </c>
       <c r="H22" s="19" t="inlineStr">
         <is>
           <t>US 60-day Iran oil waiver; 67M bbls</t>
@@ -6377,11 +7030,29 @@
       <c r="B23" s="19" t="n">
         <v>69.5</v>
       </c>
-      <c r="C23" s="19" t="n"/>
-      <c r="D23" s="19" t="n"/>
-      <c r="E23" s="19" t="n"/>
-      <c r="F23" s="19" t="n"/>
-      <c r="G23" s="19" t="n"/>
+      <c r="C23" s="19" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="D23" s="19" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E23" s="47" t="n">
+        <v>-0.0531</v>
+      </c>
+      <c r="F23" s="19" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G23" s="19" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="H23" s="19" t="inlineStr">
         <is>
           <t>WTI &lt;$70 after cargo-ship attack near Oman</t>
@@ -6394,14 +7065,30 @@
           <t>Jun 29</t>
         </is>
       </c>
-      <c r="B24" s="19" t="n"/>
+      <c r="B24" s="19" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="C24" s="19" t="n">
         <v>73.17</v>
       </c>
-      <c r="D24" s="19" t="n"/>
-      <c r="E24" s="19" t="n"/>
-      <c r="F24" s="19" t="n"/>
-      <c r="G24" s="19" t="n"/>
+      <c r="D24" s="19" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E24" s="19" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="F24" s="47" t="n">
+        <v>-0.3525</v>
+      </c>
+      <c r="G24" s="47" t="n">
+        <v>0.1115</v>
+      </c>
       <c r="H24" s="19" t="inlineStr">
         <is>
           <t>Renewed US-Iran strikes</t>
@@ -6423,9 +7110,15 @@
       <c r="D25" s="19" t="n">
         <v>2.99</v>
       </c>
-      <c r="E25" s="19" t="n"/>
-      <c r="F25" s="19" t="n"/>
-      <c r="G25" s="19" t="n"/>
+      <c r="E25" s="47" t="n">
+        <v>-0.0132</v>
+      </c>
+      <c r="F25" s="47" t="n">
+        <v>-0.0219</v>
+      </c>
+      <c r="G25" s="47" t="n">
+        <v>0.0872</v>
+      </c>
       <c r="H25" s="19" t="inlineStr">
         <is>
           <t>Iran exports surge &gt;40M bbls; &gt;10M bpd via Hormuz</t>
@@ -6447,9 +7140,15 @@
       <c r="D26" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="E26" s="19" t="n"/>
-      <c r="F26" s="19" t="n"/>
-      <c r="G26" s="19" t="n"/>
+      <c r="E26" s="47" t="n">
+        <v>-0.008500000000000001</v>
+      </c>
+      <c r="F26" s="47" t="n">
+        <v>-0.0707</v>
+      </c>
+      <c r="G26" s="47" t="n">
+        <v>0.033</v>
+      </c>
       <c r="H26" s="19" t="inlineStr">
         <is>
           <t>Crude &lt;$68 (lowest since late Feb); Brent -21% June</t>
@@ -6474,8 +7173,12 @@
       <c r="E27" s="41" t="n">
         <v>0.044</v>
       </c>
-      <c r="F27" s="41" t="n"/>
-      <c r="G27" s="41" t="n"/>
+      <c r="F27" s="45" t="n">
+        <v>0.0663</v>
+      </c>
+      <c r="G27" s="45" t="n">
+        <v>0.1852</v>
+      </c>
       <c r="H27" s="41" t="inlineStr">
         <is>
           <t>Trump declares Iran ceasefire over; WTI +4.4%, Brent +5.2%</t>
@@ -6488,12 +7191,36 @@
           <t>Jul 9</t>
         </is>
       </c>
-      <c r="B28" s="41" t="n"/>
-      <c r="C28" s="41" t="n"/>
-      <c r="D28" s="41" t="n"/>
-      <c r="E28" s="41" t="n"/>
-      <c r="F28" s="41" t="n"/>
-      <c r="G28" s="41" t="n"/>
+      <c r="B28" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="C28" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="D28" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E28" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="F28" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G28" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="H28" s="41" t="inlineStr">
         <is>
           <t>Prices ease after spike; supply-disruption fears persist</t>
@@ -6506,12 +7233,36 @@
           <t>Jul 17</t>
         </is>
       </c>
-      <c r="B29" s="41" t="n"/>
-      <c r="C29" s="41" t="n"/>
-      <c r="D29" s="41" t="n"/>
-      <c r="E29" s="41" t="n"/>
-      <c r="F29" s="41" t="n"/>
-      <c r="G29" s="41" t="n"/>
+      <c r="B29" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="C29" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="D29" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E29" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="F29" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G29" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="H29" s="41" t="inlineStr">
         <is>
           <t>Oil spikes; energy stocks rally as tech routs</t>
@@ -6524,14 +7275,30 @@
           <t>Jul 20</t>
         </is>
       </c>
-      <c r="B30" s="41" t="n"/>
+      <c r="B30" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="C30" s="41" t="n">
         <v>90</v>
       </c>
-      <c r="D30" s="41" t="n"/>
-      <c r="E30" s="41" t="n"/>
-      <c r="F30" s="41" t="n"/>
-      <c r="G30" s="41" t="n"/>
+      <c r="D30" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E30" s="41" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="F30" s="45" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="G30" s="45" t="n">
+        <v>0.3672</v>
+      </c>
       <c r="H30" s="41" t="inlineStr">
         <is>
           <t>Brent crosses $90 (+30% off July lows); Iran intercepts 4 Hormuz vessels; US resumes blockade</t>
@@ -6772,7 +7539,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>~$700B hyperscaler capex</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -6982,7 +7749,7 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -7318,7 +8085,7 @@
       </c>
       <c r="E21" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>SOX −10.3%</t>
         </is>
       </c>
       <c r="F21" s="19" t="inlineStr">
@@ -7486,7 +8253,7 @@
       </c>
       <c r="E25" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>4.25–4.50% target</t>
         </is>
       </c>
       <c r="F25" s="19" t="inlineStr">
@@ -7528,7 +8295,7 @@
       </c>
       <c r="E26" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>SMH −6.5% / KOSPI −9.99%</t>
         </is>
       </c>
       <c r="F26" s="19" t="inlineStr">
@@ -7696,7 +8463,7 @@
       </c>
       <c r="E30" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Best quarter since 2020</t>
         </is>
       </c>
       <c r="F30" s="19" t="inlineStr">
@@ -7780,7 +8547,7 @@
       </c>
       <c r="E32" s="41" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>S&amp;P +1.65%</t>
         </is>
       </c>
       <c r="F32" s="41" t="inlineStr">
@@ -7864,7 +8631,7 @@
       </c>
       <c r="E34" s="41" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>WTI $73.52 / Brent $78.02</t>
         </is>
       </c>
       <c r="F34" s="41" t="inlineStr">
@@ -7906,7 +8673,7 @@
       </c>
       <c r="E35" s="41" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Below IPO price</t>
         </is>
       </c>
       <c r="F35" s="41" t="inlineStr">
@@ -7948,7 +8715,7 @@
       </c>
       <c r="E36" s="41" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Nasdaq week −2.90%</t>
         </is>
       </c>
       <c r="F36" s="41" t="inlineStr">
@@ -8067,7 +8834,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A48"/>
+  <dimension ref="A1:A53"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.609375" defaultRowHeight="15"/>
   <cols>
     <col width="89.99609375" customWidth="1" style="37" min="1" max="1"/>
@@ -8358,11 +9125,38 @@
         </is>
       </c>
     </row>
-    <row r="47"/>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
           <t>- MA/MTD% values computed at finalization (static values; environment could not run a live recalc engine).</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Blank-cell fill pass (2026-07-21):</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>- Oil: spread = Brent−WTI; WTI Δ% vs prior LOGGED print; Brent MTD% baselines Apr/102.00, May/107.80 (Apr 30), Jun/113.00 (May 15, last logged), Jul/73.17 (Jun 29, last logged); Brent YoY vs 65.83 constant (original sheet convention).</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>- 'n/d' = print not published in available sources — explicitly flagged, never fabricated. '—' = no signal that day.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>- S&amp;P Daily Δ / Δ% across source gaps computed vs prior LOGGED close (May 6, May 11, May 14, Jun 4, Jun 5, Jun 17 etc.).</t>
         </is>
       </c>
     </row>

</xml_diff>